<commit_message>
adjust the condition to colour and the wording arrangemnet of 6months
</commit_message>
<xml_diff>
--- a/Knockout Matrix Template_FILLED.xlsx
+++ b/Knockout Matrix Template_FILLED.xlsx
@@ -138,7 +138,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -169,6 +169,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
+        <bgColor rgb="00FFFF00"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="24">
     <border>
@@ -431,7 +437,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="134">
+  <cellXfs count="138">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -750,6 +756,16 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1293,7 +1309,7 @@
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>GREATOCEAN AUTOMOBILE SUPPLY SDN. BHD.</t>
+          <t>NBRAND (M) SDN. BHD.</t>
         </is>
       </c>
       <c r="F6" s="8" t="n"/>
@@ -1348,7 +1364,7 @@
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
-          <t>2025-12-16</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="K7" s="8" t="n"/>
@@ -1359,13 +1375,26 @@
       </c>
       <c r="M7" s="12" t="inlineStr">
         <is>
-          <t>GREATOCEAN AUTOMOBILE SUPPLY SDN. BHD.</t>
+          <t>NBRAND (M) SDN. BHD.</t>
         </is>
       </c>
       <c r="N7" s="5" t="n"/>
-      <c r="O7" s="13" t="n"/>
+      <c r="O7" s="13" t="inlineStr">
+        <is>
+          <t>SIEW WAI FEN</t>
+        </is>
+      </c>
       <c r="P7" s="5" t="n"/>
-      <c r="Q7" s="13" t="n"/>
+      <c r="Q7" s="13" t="inlineStr">
+        <is>
+          <t>TEOH CHUN AIK</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>TEOH YONYEW</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="17.1" customFormat="1" customHeight="1" s="2">
       <c r="D8" s="6" t="inlineStr">
@@ -1453,19 +1482,24 @@
       <c r="L11" s="17" t="n"/>
       <c r="M11" s="18" t="inlineStr">
         <is>
-          <t>678</t>
+          <t>750</t>
         </is>
       </c>
       <c r="N11" s="5" t="n"/>
       <c r="O11" s="18" t="inlineStr">
         <is>
-          <t>311</t>
+          <t>648</t>
         </is>
       </c>
       <c r="P11" s="5" t="n"/>
       <c r="Q11" s="18" t="inlineStr">
         <is>
-          <t>533</t>
+          <t>640</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>570</t>
         </is>
       </c>
       <c r="V11" s="19" t="inlineStr">
@@ -1501,19 +1535,24 @@
       </c>
       <c r="M12" s="18" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="N12" s="5" t="n"/>
       <c r="O12" s="18" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="P12" s="5" t="n"/>
       <c r="Q12" s="18" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="V12" s="19" t="inlineStr">
@@ -1547,7 +1586,7 @@
       </c>
       <c r="M13" s="23" t="inlineStr">
         <is>
-          <t>2011</t>
+          <t>2014</t>
         </is>
       </c>
       <c r="N13" s="5" t="n"/>
@@ -1726,7 +1765,7 @@
       </c>
       <c r="M18" s="18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N18" s="5" t="n"/>
@@ -1738,7 +1777,12 @@
       <c r="P18" s="5" t="n"/>
       <c r="Q18" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>5</t>
         </is>
       </c>
     </row>
@@ -1774,6 +1818,11 @@
       <c r="P19" s="5" t="n"/>
       <c r="Q19" s="18" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
@@ -1813,6 +1862,11 @@
           <t>0</t>
         </is>
       </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="17.1" customFormat="1" customHeight="1" s="2">
       <c r="D21" s="115" t="inlineStr">
@@ -1834,19 +1888,24 @@
       </c>
       <c r="M21" s="18" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>11</t>
         </is>
       </c>
       <c r="N21" s="5" t="n"/>
       <c r="O21" s="18" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="P21" s="5" t="n"/>
       <c r="Q21" s="18" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>5</t>
         </is>
       </c>
     </row>
@@ -1868,9 +1927,9 @@
           <t>≥1</t>
         </is>
       </c>
-      <c r="M22" s="18" t="inlineStr">
-        <is>
-          <t>0</t>
+      <c r="M22" s="130" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
       <c r="N22" s="5" t="n"/>
@@ -1881,6 +1940,11 @@
       </c>
       <c r="P22" s="5" t="n"/>
       <c r="Q22" s="18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -1904,9 +1968,9 @@
           <t>Subject as "Defendant" and case is "Ongoing" only</t>
         </is>
       </c>
-      <c r="M23" s="27" t="inlineStr">
-        <is>
-          <t>No, No, No</t>
+      <c r="M23" s="131" t="inlineStr">
+        <is>
+          <t>Yes, No, No</t>
         </is>
       </c>
       <c r="N23" s="5" t="n"/>
@@ -1917,6 +1981,11 @@
       </c>
       <c r="P23" s="5" t="n"/>
       <c r="Q23" s="27" t="inlineStr">
+        <is>
+          <t>No, No, No</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
         <is>
           <t>No, No, No</t>
         </is>
@@ -1972,11 +2041,16 @@
       <c r="N25" s="5" t="n"/>
       <c r="O25" s="18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="P25" s="5" t="n"/>
       <c r="Q25" s="18" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -2017,6 +2091,11 @@
           <t>0</t>
         </is>
       </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="20.1" customFormat="1" customHeight="1" s="2">
       <c r="D27" s="115" t="inlineStr">
@@ -2038,19 +2117,24 @@
       </c>
       <c r="M27" s="28" t="inlineStr">
         <is>
-          <t>15436493</t>
+          <t>3448225</t>
         </is>
       </c>
       <c r="N27" s="5" t="n"/>
       <c r="O27" s="28" t="inlineStr">
         <is>
-          <t>1753657</t>
+          <t>3448225</t>
         </is>
       </c>
       <c r="P27" s="5" t="n"/>
       <c r="Q27" s="28" t="inlineStr">
         <is>
-          <t>1723015</t>
+          <t>3448225</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>3448225</t>
         </is>
       </c>
     </row>
@@ -2074,19 +2158,24 @@
       </c>
       <c r="M28" s="28" t="inlineStr">
         <is>
-          <t>16364987</t>
+          <t>5316000</t>
         </is>
       </c>
       <c r="N28" s="5" t="n"/>
       <c r="O28" s="28" t="inlineStr">
         <is>
-          <t>2146309</t>
+          <t>5316000</t>
         </is>
       </c>
       <c r="P28" s="5" t="n"/>
       <c r="Q28" s="28" t="inlineStr">
         <is>
-          <t>2094126</t>
+          <t>5316000</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>5316000</t>
         </is>
       </c>
     </row>
@@ -2110,19 +2199,24 @@
       </c>
       <c r="M29" s="28" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="N29" s="5" t="n"/>
       <c r="O29" s="24" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="P29" s="5" t="n"/>
       <c r="Q29" s="24" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>YES, outstanding: 4983453.0, limit: 5000000.0</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -2146,19 +2240,24 @@
       </c>
       <c r="M30" s="28" t="inlineStr">
         <is>
-          <t>YES, outstanding: 15520690.0, limit: 17714987.0</t>
+          <t>YES, outstanding: 3448225.0, limit: 5316000.0</t>
         </is>
       </c>
       <c r="N30" s="5" t="n"/>
       <c r="O30" s="24" t="inlineStr">
         <is>
-          <t>YES, outstanding: 15520690.0, limit: 17714987.0</t>
+          <t>YES, outstanding: 3448225.0, limit: 5316000.0</t>
         </is>
       </c>
       <c r="P30" s="5" t="n"/>
       <c r="Q30" s="24" t="inlineStr">
         <is>
-          <t>YES, outstanding: 15520690.0, limit: 17714987.0</t>
+          <t>YES, outstanding: 3448225.0, limit: 5316000.0</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>YES, outstanding: 3448225.0, limit: 5316000.0</t>
         </is>
       </c>
     </row>
@@ -2182,19 +2281,24 @@
       </c>
       <c r="M31" s="27" t="inlineStr">
         <is>
-          <t>current 1 month MIA1: 1, MIA2: 0, MIA3: 0, MIA4+: 0 and /or past 6 months MIA1: 1, MIA2: 0, MIA3: 0, MIA4+: 0</t>
+          <t>past 6 months MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 0 and /or current 1 month MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 0</t>
         </is>
       </c>
       <c r="N31" s="5" t="n"/>
       <c r="O31" s="27" t="inlineStr">
         <is>
-          <t>current 1 month MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 1 and /or past 6 months MIA1: 1, MIA2: 1, MIA3: 1, MIA4+: 2</t>
+          <t>past 6 months MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 0 and /or current 1 month MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 0</t>
         </is>
       </c>
       <c r="P31" s="5" t="n"/>
       <c r="Q31" s="27" t="inlineStr">
         <is>
-          <t>current 1 month MIA1: 0, MIA2: 1, MIA3: 0, MIA4+: 0 and /or past 6 months MIA1: 6, MIA2: 3, MIA3: 1, MIA4+: 0</t>
+          <t>past 6 months MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 0 and /or current 1 month MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 0</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>past 6 months MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 0 and /or current 1 month MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 0</t>
         </is>
       </c>
     </row>
@@ -2240,19 +2344,24 @@
           <t>No</t>
         </is>
       </c>
-      <c r="M33" s="28" t="inlineStr">
+      <c r="M33" s="132" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
       <c r="N33" s="5" t="n"/>
-      <c r="O33" s="24" t="inlineStr">
+      <c r="O33" s="131" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
       <c r="P33" s="5" t="n"/>
-      <c r="Q33" s="24" t="inlineStr">
+      <c r="Q33" s="131" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="S33" s="133" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -2278,19 +2387,24 @@
       </c>
       <c r="M34" s="27" t="inlineStr">
         <is>
-          <t>current 1 month MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 0 and /or past 6 months MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 0</t>
+          <t>past 6 months MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 0 and /or current 1 month MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 0</t>
         </is>
       </c>
       <c r="N34" s="5" t="n"/>
       <c r="O34" s="27" t="inlineStr">
         <is>
-          <t>current 1 month MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 0 and /or past 6 months MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 0</t>
+          <t>past 6 months MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 0 and /or current 1 month MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 0</t>
         </is>
       </c>
       <c r="P34" s="5" t="n"/>
       <c r="Q34" s="27" t="inlineStr">
         <is>
-          <t>current 1 month MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 0 and /or past 6 months MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 0</t>
+          <t>past 6 months MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 0 and /or current 1 month MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 0</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>past 6 months MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 0 and /or current 1 month MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 0</t>
         </is>
       </c>
     </row>
@@ -2312,19 +2426,24 @@
           <t>Any positive notation</t>
         </is>
       </c>
-      <c r="M35" s="18" t="inlineStr">
+      <c r="M35" s="130" t="inlineStr">
         <is>
           <t>WITHDRAWN</t>
         </is>
       </c>
       <c r="N35" s="5" t="n"/>
-      <c r="O35" s="27" t="inlineStr">
+      <c r="O35" s="131" t="inlineStr">
         <is>
           <t>WITHDRAWN</t>
         </is>
       </c>
       <c r="P35" s="5" t="n"/>
-      <c r="Q35" s="27" t="inlineStr">
+      <c r="Q35" s="131" t="inlineStr">
+        <is>
+          <t>WITHDRAWN</t>
+        </is>
+      </c>
+      <c r="S35" s="133" t="inlineStr">
         <is>
           <t>WITHDRAWN</t>
         </is>
@@ -2541,7 +2660,7 @@
       <c r="L44" s="36" t="n"/>
     </row>
     <row r="45">
-      <c r="D45" s="130" t="n"/>
+      <c r="D45" s="134" t="n"/>
       <c r="H45" s="34" t="n"/>
       <c r="I45" s="35" t="n"/>
       <c r="J45" s="34" t="n"/>
@@ -2784,36 +2903,36 @@
     </row>
     <row r="58" ht="17.1" customFormat="1" customHeight="1" s="36">
       <c r="C58" s="58" t="n"/>
-      <c r="D58" s="131" t="inlineStr">
+      <c r="D58" s="135" t="inlineStr">
         <is>
           <t>By Credit Analyst</t>
         </is>
       </c>
-      <c r="E58" s="132" t="n"/>
-      <c r="F58" s="131" t="inlineStr">
+      <c r="E58" s="136" t="n"/>
+      <c r="F58" s="135" t="inlineStr">
         <is>
           <t>Justifications:</t>
         </is>
       </c>
-      <c r="G58" s="133" t="n"/>
-      <c r="H58" s="133" t="n"/>
-      <c r="I58" s="133" t="n"/>
-      <c r="J58" s="133" t="n"/>
-      <c r="K58" s="132" t="n"/>
+      <c r="G58" s="137" t="n"/>
+      <c r="H58" s="137" t="n"/>
+      <c r="I58" s="137" t="n"/>
+      <c r="J58" s="137" t="n"/>
+      <c r="K58" s="136" t="n"/>
       <c r="L58" s="63" t="inlineStr">
         <is>
           <t>By Chief Credit Officer</t>
         </is>
       </c>
-      <c r="M58" s="131" t="inlineStr">
+      <c r="M58" s="135" t="inlineStr">
         <is>
           <t>Justifications:</t>
         </is>
       </c>
-      <c r="N58" s="133" t="n"/>
-      <c r="O58" s="133" t="n"/>
-      <c r="P58" s="133" t="n"/>
-      <c r="Q58" s="132" t="n"/>
+      <c r="N58" s="137" t="n"/>
+      <c r="O58" s="137" t="n"/>
+      <c r="P58" s="137" t="n"/>
+      <c r="Q58" s="136" t="n"/>
       <c r="R58" s="57" t="n"/>
       <c r="S58" s="1" t="n"/>
     </row>
@@ -2969,36 +3088,36 @@
     </row>
     <row r="67" ht="14.25" customFormat="1" customHeight="1" s="36">
       <c r="C67" s="58" t="n"/>
-      <c r="D67" s="131" t="inlineStr">
+      <c r="D67" s="135" t="inlineStr">
         <is>
           <t>By Credit Committee 1</t>
         </is>
       </c>
-      <c r="E67" s="132" t="n"/>
-      <c r="F67" s="131" t="inlineStr">
+      <c r="E67" s="136" t="n"/>
+      <c r="F67" s="135" t="inlineStr">
         <is>
           <t>Justifications:</t>
         </is>
       </c>
-      <c r="G67" s="133" t="n"/>
-      <c r="H67" s="133" t="n"/>
-      <c r="I67" s="133" t="n"/>
-      <c r="J67" s="133" t="n"/>
-      <c r="K67" s="132" t="n"/>
+      <c r="G67" s="137" t="n"/>
+      <c r="H67" s="137" t="n"/>
+      <c r="I67" s="137" t="n"/>
+      <c r="J67" s="137" t="n"/>
+      <c r="K67" s="136" t="n"/>
       <c r="L67" s="78" t="inlineStr">
         <is>
           <t>By Credit Committee 2</t>
         </is>
       </c>
-      <c r="M67" s="131" t="inlineStr">
+      <c r="M67" s="135" t="inlineStr">
         <is>
           <t>Justifications:</t>
         </is>
       </c>
-      <c r="N67" s="133" t="n"/>
-      <c r="O67" s="133" t="n"/>
-      <c r="P67" s="133" t="n"/>
-      <c r="Q67" s="132" t="n"/>
+      <c r="N67" s="137" t="n"/>
+      <c r="O67" s="137" t="n"/>
+      <c r="P67" s="137" t="n"/>
+      <c r="Q67" s="136" t="n"/>
       <c r="R67" s="57" t="n"/>
       <c r="S67" s="1" t="n"/>
     </row>

</xml_diff>

<commit_message>
Remove the record num
</commit_message>
<xml_diff>
--- a/Knockout Matrix Template_FILLED.xlsx
+++ b/Knockout Matrix Template_FILLED.xlsx
@@ -31,7 +31,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]d\-mmm\-yy;@"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -137,8 +137,12 @@
       <b val="1"/>
       <sz val="12"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FF0000"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -169,12 +173,6 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
-        <bgColor rgb="00FFFF00"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="24">
     <border>
@@ -753,19 +751,21 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1309,7 +1309,7 @@
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>NBRAND (M) SDN. BHD.</t>
+          <t>GREATOCEAN AUTOMOBILE SUPPLY SDN. BHD.</t>
         </is>
       </c>
       <c r="F6" s="8" t="n"/>
@@ -1364,7 +1364,7 @@
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2025-12-16</t>
         </is>
       </c>
       <c r="K7" s="8" t="n"/>
@@ -1375,24 +1375,19 @@
       </c>
       <c r="M7" s="12" t="inlineStr">
         <is>
-          <t>NBRAND (M) SDN. BHD.</t>
+          <t>GREATOCEAN AUTOMOBILE SUPPLY SDN. BHD.</t>
         </is>
       </c>
       <c r="N7" s="5" t="n"/>
       <c r="O7" s="13" t="inlineStr">
         <is>
-          <t>SIEW WAI FEN</t>
+          <t>CHING SOO YING</t>
         </is>
       </c>
       <c r="P7" s="5" t="n"/>
       <c r="Q7" s="13" t="inlineStr">
         <is>
-          <t>TEOH CHUN AIK</t>
-        </is>
-      </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>TEOH YONYEW</t>
+          <t>LIM JUN YEONG</t>
         </is>
       </c>
     </row>
@@ -1482,24 +1477,19 @@
       <c r="L11" s="17" t="n"/>
       <c r="M11" s="18" t="inlineStr">
         <is>
-          <t>750</t>
+          <t>678</t>
         </is>
       </c>
       <c r="N11" s="5" t="n"/>
       <c r="O11" s="18" t="inlineStr">
         <is>
-          <t>648</t>
+          <t>311</t>
         </is>
       </c>
       <c r="P11" s="5" t="n"/>
       <c r="Q11" s="18" t="inlineStr">
         <is>
-          <t>640</t>
-        </is>
-      </c>
-      <c r="S11" t="inlineStr">
-        <is>
-          <t>570</t>
+          <t>533</t>
         </is>
       </c>
       <c r="V11" s="19" t="inlineStr">
@@ -1535,24 +1525,19 @@
       </c>
       <c r="M12" s="18" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="N12" s="5" t="n"/>
-      <c r="O12" s="18" t="inlineStr">
-        <is>
-          <t>B</t>
+      <c r="O12" s="129" t="inlineStr">
+        <is>
+          <t>F</t>
         </is>
       </c>
       <c r="P12" s="5" t="n"/>
       <c r="Q12" s="18" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="S12" t="inlineStr">
-        <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="V12" s="19" t="inlineStr">
@@ -1566,7 +1551,7 @@
       </c>
     </row>
     <row r="13" ht="33.95" customFormat="1" customHeight="1" s="2">
-      <c r="D13" s="129" t="inlineStr">
+      <c r="D13" s="130" t="inlineStr">
         <is>
           <t>Business has been in operations for at least THREE (3) years (Including upgrade from Sole Proprietorship and Partnership under similar business activity)</t>
         </is>
@@ -1586,7 +1571,7 @@
       </c>
       <c r="M13" s="23" t="inlineStr">
         <is>
-          <t>2014</t>
+          <t>2,011</t>
         </is>
       </c>
       <c r="N13" s="5" t="n"/>
@@ -1608,7 +1593,7 @@
       </c>
     </row>
     <row r="14" ht="17.1" customFormat="1" customHeight="1" s="2">
-      <c r="D14" s="129" t="inlineStr">
+      <c r="D14" s="130" t="inlineStr">
         <is>
           <t>Key Directors must have at least 3 years involvement in the business and/or relevant related industries.</t>
         </is>
@@ -1746,7 +1731,7 @@
       <c r="Q17" s="18" t="n"/>
     </row>
     <row r="18" ht="17.1" customFormat="1" customHeight="1" s="2">
-      <c r="D18" s="129" t="inlineStr">
+      <c r="D18" s="130" t="inlineStr">
         <is>
           <t>Credit Applications Approved for Last 12 months (per primary CRA report)</t>
         </is>
@@ -1765,7 +1750,7 @@
       </c>
       <c r="M18" s="18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N18" s="5" t="n"/>
@@ -1777,17 +1762,12 @@
       <c r="P18" s="5" t="n"/>
       <c r="Q18" s="18" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="S18" t="inlineStr">
-        <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="19" ht="33.95" customFormat="1" customHeight="1" s="2">
-      <c r="D19" s="129" t="inlineStr">
+      <c r="D19" s="130" t="inlineStr">
         <is>
           <t>Credit Applications Pending (per primary CRA report)</t>
         </is>
@@ -1818,11 +1798,6 @@
       <c r="P19" s="5" t="n"/>
       <c r="Q19" s="18" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="S19" t="inlineStr">
-        <is>
           <t>0</t>
         </is>
       </c>
@@ -1862,11 +1837,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="S20" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
     </row>
     <row r="21" ht="17.1" customFormat="1" customHeight="1" s="2">
       <c r="D21" s="115" t="inlineStr">
@@ -1888,24 +1858,19 @@
       </c>
       <c r="M21" s="18" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>16</t>
         </is>
       </c>
       <c r="N21" s="5" t="n"/>
       <c r="O21" s="18" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="P21" s="5" t="n"/>
       <c r="Q21" s="18" t="inlineStr">
         <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="S21" t="inlineStr">
-        <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
     </row>
@@ -1927,9 +1892,9 @@
           <t>≥1</t>
         </is>
       </c>
-      <c r="M22" s="130" t="inlineStr">
-        <is>
-          <t>3</t>
+      <c r="M22" s="18" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
       <c r="N22" s="5" t="n"/>
@@ -1940,11 +1905,6 @@
       </c>
       <c r="P22" s="5" t="n"/>
       <c r="Q22" s="18" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="S22" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -1968,9 +1928,9 @@
           <t>Subject as "Defendant" and case is "Ongoing" only</t>
         </is>
       </c>
-      <c r="M23" s="131" t="inlineStr">
-        <is>
-          <t>Yes, No, No</t>
+      <c r="M23" s="27" t="inlineStr">
+        <is>
+          <t>No, No, No</t>
         </is>
       </c>
       <c r="N23" s="5" t="n"/>
@@ -1981,11 +1941,6 @@
       </c>
       <c r="P23" s="5" t="n"/>
       <c r="Q23" s="27" t="inlineStr">
-        <is>
-          <t>No, No, No</t>
-        </is>
-      </c>
-      <c r="S23" t="inlineStr">
         <is>
           <t>No, No, No</t>
         </is>
@@ -2041,16 +1996,11 @@
       <c r="N25" s="5" t="n"/>
       <c r="O25" s="18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="P25" s="5" t="n"/>
       <c r="Q25" s="18" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="S25" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -2091,11 +2041,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="S26" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
     </row>
     <row r="27" ht="20.1" customFormat="1" customHeight="1" s="2">
       <c r="D27" s="115" t="inlineStr">
@@ -2117,24 +2062,19 @@
       </c>
       <c r="M27" s="28" t="inlineStr">
         <is>
-          <t>3448225</t>
+          <t>18,997,362</t>
         </is>
       </c>
       <c r="N27" s="5" t="n"/>
       <c r="O27" s="28" t="inlineStr">
         <is>
-          <t>3448225</t>
+          <t>18,997,362</t>
         </is>
       </c>
       <c r="P27" s="5" t="n"/>
       <c r="Q27" s="28" t="inlineStr">
         <is>
-          <t>3448225</t>
-        </is>
-      </c>
-      <c r="S27" t="inlineStr">
-        <is>
-          <t>3448225</t>
+          <t>18,997,362</t>
         </is>
       </c>
     </row>
@@ -2158,24 +2098,19 @@
       </c>
       <c r="M28" s="28" t="inlineStr">
         <is>
-          <t>5316000</t>
+          <t>21,955,422</t>
         </is>
       </c>
       <c r="N28" s="5" t="n"/>
       <c r="O28" s="28" t="inlineStr">
         <is>
-          <t>5316000</t>
+          <t>21,955,422</t>
         </is>
       </c>
       <c r="P28" s="5" t="n"/>
       <c r="Q28" s="28" t="inlineStr">
         <is>
-          <t>5316000</t>
-        </is>
-      </c>
-      <c r="S28" t="inlineStr">
-        <is>
-          <t>5316000</t>
+          <t>21,955,422</t>
         </is>
       </c>
     </row>
@@ -2199,7 +2134,7 @@
       </c>
       <c r="M29" s="28" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>YES, outstanding: 1,451,424, limit: 1,500,000</t>
         </is>
       </c>
       <c r="N29" s="5" t="n"/>
@@ -2210,11 +2145,6 @@
       </c>
       <c r="P29" s="5" t="n"/>
       <c r="Q29" s="24" t="inlineStr">
-        <is>
-          <t>YES, outstanding: 4983453.0, limit: 5000000.0</t>
-        </is>
-      </c>
-      <c r="S29" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -2240,24 +2170,19 @@
       </c>
       <c r="M30" s="28" t="inlineStr">
         <is>
-          <t>YES, outstanding: 3448225.0, limit: 5316000.0</t>
+          <t>16: YES, outstanding: 15,520,690, limit: 17,714,987</t>
         </is>
       </c>
       <c r="N30" s="5" t="n"/>
       <c r="O30" s="24" t="inlineStr">
         <is>
-          <t>YES, outstanding: 3448225.0, limit: 5316000.0</t>
+          <t>10: YES, outstanding: 1,753,657, limit: 2,146,309</t>
         </is>
       </c>
       <c r="P30" s="5" t="n"/>
       <c r="Q30" s="24" t="inlineStr">
         <is>
-          <t>YES, outstanding: 3448225.0, limit: 5316000.0</t>
-        </is>
-      </c>
-      <c r="S30" t="inlineStr">
-        <is>
-          <t>YES, outstanding: 3448225.0, limit: 5316000.0</t>
+          <t>9: YES, outstanding: 1,723,015, limit: 2,094,126</t>
         </is>
       </c>
     </row>
@@ -2281,24 +2206,19 @@
       </c>
       <c r="M31" s="27" t="inlineStr">
         <is>
-          <t>past 6 months MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 0 and /or current 1 month MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 0</t>
+          <t>past 6 months MIA1: 1, MIA2: 0, MIA3: 0, MIA4+: 0 and /or current 1 month MIA1: 1, MIA2: 0, MIA3: 0, MIA4+: 0</t>
         </is>
       </c>
       <c r="N31" s="5" t="n"/>
-      <c r="O31" s="27" t="inlineStr">
-        <is>
-          <t>past 6 months MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 0 and /or current 1 month MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 0</t>
+      <c r="O31" s="131" t="inlineStr">
+        <is>
+          <t>past 6 months MIA1: 1, MIA2: 1, MIA3: 1, MIA4+: 2 and /or current 1 month MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 1</t>
         </is>
       </c>
       <c r="P31" s="5" t="n"/>
-      <c r="Q31" s="27" t="inlineStr">
-        <is>
-          <t>past 6 months MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 0 and /or current 1 month MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 0</t>
-        </is>
-      </c>
-      <c r="S31" t="inlineStr">
-        <is>
-          <t>past 6 months MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 0 and /or current 1 month MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 0</t>
+      <c r="Q31" s="131" t="inlineStr">
+        <is>
+          <t>past 6 months MIA1: 6, MIA2: 3, MIA3: 1, MIA4+: 0 and /or current 1 month MIA1: 0, MIA2: 1, MIA3: 0, MIA4+: 0</t>
         </is>
       </c>
     </row>
@@ -2320,11 +2240,23 @@
           <t>Any positive notation</t>
         </is>
       </c>
-      <c r="M32" s="18" t="n"/>
+      <c r="M32" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="N32" s="5" t="n"/>
-      <c r="O32" s="18" t="n"/>
+      <c r="O32" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="P32" s="5" t="n"/>
-      <c r="Q32" s="18" t="n"/>
+      <c r="Q32" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="42" customFormat="1" customHeight="1" s="2">
       <c r="D33" s="115" t="inlineStr">
@@ -2350,18 +2282,13 @@
         </is>
       </c>
       <c r="N33" s="5" t="n"/>
-      <c r="O33" s="131" t="inlineStr">
+      <c r="O33" s="133" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
       <c r="P33" s="5" t="n"/>
-      <c r="Q33" s="131" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="S33" s="133" t="inlineStr">
+      <c r="Q33" s="133" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -2387,24 +2314,19 @@
       </c>
       <c r="M34" s="27" t="inlineStr">
         <is>
-          <t>past 6 months MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 0 and /or current 1 month MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 0</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="N34" s="5" t="n"/>
       <c r="O34" s="27" t="inlineStr">
         <is>
-          <t>past 6 months MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 0 and /or current 1 month MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 0</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="P34" s="5" t="n"/>
       <c r="Q34" s="27" t="inlineStr">
         <is>
-          <t>past 6 months MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 0 and /or current 1 month MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 0</t>
-        </is>
-      </c>
-      <c r="S34" t="inlineStr">
-        <is>
-          <t>past 6 months MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 0 and /or current 1 month MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 0</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2348,7 @@
           <t>Any positive notation</t>
         </is>
       </c>
-      <c r="M35" s="130" t="inlineStr">
+      <c r="M35" s="129" t="inlineStr">
         <is>
           <t>WITHDRAWN</t>
         </is>
@@ -2443,14 +2365,9 @@
           <t>WITHDRAWN</t>
         </is>
       </c>
-      <c r="S35" s="133" t="inlineStr">
-        <is>
-          <t>WITHDRAWN</t>
-        </is>
-      </c>
     </row>
     <row r="36" ht="33.95" customFormat="1" customHeight="1" s="2">
-      <c r="D36" s="129" t="inlineStr">
+      <c r="D36" s="130" t="inlineStr">
         <is>
           <t>Issuer must be profitable for at least TWO (2) out of THREE (3) years with the most recent years showing profit (From either Primary CRA Report / SSM / Audited Report /Draft Audited Report)</t>
         </is>
@@ -2482,7 +2399,7 @@
       </c>
     </row>
     <row r="37" ht="36.75" customFormat="1" customHeight="1" s="2">
-      <c r="D37" s="129" t="inlineStr">
+      <c r="D37" s="130" t="inlineStr">
         <is>
           <t>Positive Networth in latest FYE (From either Primary CRA Report / SSM / Audited Report /Draft Audited Report)</t>
         </is>

</xml_diff>

<commit_message>
Code redundancy fixed version 1
</commit_message>
<xml_diff>
--- a/Knockout Matrix Template_FILLED.xlsx
+++ b/Knockout Matrix Template_FILLED.xlsx
@@ -435,7 +435,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="138">
+  <cellXfs count="139">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -760,6 +760,7 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1309,7 +1310,7 @@
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>GREATOCEAN AUTOMOBILE SUPPLY SDN. BHD.</t>
+          <t>EVER FRESH CAMERON SDN. BHD.</t>
         </is>
       </c>
       <c r="F6" s="8" t="n"/>
@@ -1364,7 +1365,7 @@
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
-          <t>2025-12-16</t>
+          <t>2025-10-28</t>
         </is>
       </c>
       <c r="K7" s="8" t="n"/>
@@ -1375,19 +1376,29 @@
       </c>
       <c r="M7" s="12" t="inlineStr">
         <is>
-          <t>GREATOCEAN AUTOMOBILE SUPPLY SDN. BHD.</t>
+          <t>EVER FRESH CAMERON SDN. BHD.</t>
         </is>
       </c>
       <c r="N7" s="5" t="n"/>
       <c r="O7" s="13" t="inlineStr">
         <is>
-          <t>CHING SOO YING</t>
+          <t>LAU HEE WOOI</t>
         </is>
       </c>
       <c r="P7" s="5" t="n"/>
       <c r="Q7" s="13" t="inlineStr">
         <is>
-          <t>LIM JUN YEONG</t>
+          <t>LAU HOOI MENG</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>LOH POEY CHUAN</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>LOH POEY CHUAN</t>
         </is>
       </c>
     </row>
@@ -1477,19 +1488,29 @@
       <c r="L11" s="17" t="n"/>
       <c r="M11" s="18" t="inlineStr">
         <is>
-          <t>678</t>
+          <t>300</t>
         </is>
       </c>
       <c r="N11" s="5" t="n"/>
       <c r="O11" s="18" t="inlineStr">
         <is>
-          <t>311</t>
+          <t>543</t>
         </is>
       </c>
       <c r="P11" s="5" t="n"/>
       <c r="Q11" s="18" t="inlineStr">
         <is>
-          <t>533</t>
+          <t>644</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>575</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>575</t>
         </is>
       </c>
       <c r="V11" s="19" t="inlineStr">
@@ -1523,21 +1544,31 @@
           <t>No Score , E or worse</t>
         </is>
       </c>
-      <c r="M12" s="18" t="inlineStr">
-        <is>
-          <t>B</t>
+      <c r="M12" s="129" t="inlineStr">
+        <is>
+          <t>F</t>
         </is>
       </c>
       <c r="N12" s="5" t="n"/>
-      <c r="O12" s="129" t="inlineStr">
-        <is>
-          <t>F</t>
+      <c r="O12" s="18" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="P12" s="5" t="n"/>
       <c r="Q12" s="18" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="V12" s="19" t="inlineStr">
@@ -1571,7 +1602,7 @@
       </c>
       <c r="M13" s="23" t="inlineStr">
         <is>
-          <t>2,011</t>
+          <t>2,013</t>
         </is>
       </c>
       <c r="N13" s="5" t="n"/>
@@ -1750,19 +1781,29 @@
       </c>
       <c r="M18" s="18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N18" s="5" t="n"/>
       <c r="O18" s="18" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
       <c r="P18" s="5" t="n"/>
       <c r="Q18" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -1801,6 +1842,16 @@
           <t>0</t>
         </is>
       </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="17.1" customFormat="1" customHeight="1" s="2">
       <c r="D20" s="115" t="inlineStr">
@@ -1837,6 +1888,16 @@
           <t>0</t>
         </is>
       </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="17.1" customFormat="1" customHeight="1" s="2">
       <c r="D21" s="115" t="inlineStr">
@@ -1858,19 +1919,29 @@
       </c>
       <c r="M21" s="18" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>35</t>
         </is>
       </c>
       <c r="N21" s="5" t="n"/>
       <c r="O21" s="18" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="P21" s="5" t="n"/>
       <c r="Q21" s="18" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -1892,9 +1963,9 @@
           <t>≥1</t>
         </is>
       </c>
-      <c r="M22" s="18" t="inlineStr">
-        <is>
-          <t>0</t>
+      <c r="M22" s="129" t="inlineStr">
+        <is>
+          <t>2</t>
         </is>
       </c>
       <c r="N22" s="5" t="n"/>
@@ -1905,6 +1976,16 @@
       </c>
       <c r="P22" s="5" t="n"/>
       <c r="Q22" s="18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -1928,9 +2009,9 @@
           <t>Subject as "Defendant" and case is "Ongoing" only</t>
         </is>
       </c>
-      <c r="M23" s="27" t="inlineStr">
-        <is>
-          <t>No, No, No</t>
+      <c r="M23" s="131" t="inlineStr">
+        <is>
+          <t>Yes, Yes, No</t>
         </is>
       </c>
       <c r="N23" s="5" t="n"/>
@@ -1941,6 +2022,16 @@
       </c>
       <c r="P23" s="5" t="n"/>
       <c r="Q23" s="27" t="inlineStr">
+        <is>
+          <t>No, No, No</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>No, No, No</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
         <is>
           <t>No, No, No</t>
         </is>
@@ -1964,11 +2055,33 @@
           <t>&gt;1 &amp; outstanding &gt;RM10k</t>
         </is>
       </c>
-      <c r="M24" s="18" t="n"/>
+      <c r="M24" s="129" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="N24" s="5" t="n"/>
-      <c r="O24" s="18" t="n"/>
+      <c r="O24" s="129" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="P24" s="5" t="n"/>
-      <c r="Q24" s="18" t="n"/>
+      <c r="Q24" s="129" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="S24" s="132" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="U24" s="132" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="17.1" customFormat="1" customHeight="1" s="2">
       <c r="D25" s="115" t="inlineStr">
@@ -1988,19 +2101,29 @@
           <t>&gt;5 per month</t>
         </is>
       </c>
-      <c r="M25" s="18" t="inlineStr">
-        <is>
-          <t>4</t>
+      <c r="M25" s="129" t="inlineStr">
+        <is>
+          <t>9</t>
         </is>
       </c>
       <c r="N25" s="5" t="n"/>
       <c r="O25" s="18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="P25" s="5" t="n"/>
       <c r="Q25" s="18" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -2041,6 +2164,16 @@
           <t>0</t>
         </is>
       </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="20.1" customFormat="1" customHeight="1" s="2">
       <c r="D27" s="115" t="inlineStr">
@@ -2062,19 +2195,29 @@
       </c>
       <c r="M27" s="28" t="inlineStr">
         <is>
-          <t>18,997,362</t>
+          <t>30,667,835</t>
         </is>
       </c>
       <c r="N27" s="5" t="n"/>
       <c r="O27" s="28" t="inlineStr">
         <is>
-          <t>18,997,362</t>
+          <t>1,349,839</t>
         </is>
       </c>
       <c r="P27" s="5" t="n"/>
       <c r="Q27" s="28" t="inlineStr">
         <is>
-          <t>18,997,362</t>
+          <t>1,278,562</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>17,053</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>17,053</t>
         </is>
       </c>
     </row>
@@ -2098,19 +2241,29 @@
       </c>
       <c r="M28" s="28" t="inlineStr">
         <is>
-          <t>21,955,422</t>
+          <t>34,070,376</t>
         </is>
       </c>
       <c r="N28" s="5" t="n"/>
       <c r="O28" s="28" t="inlineStr">
         <is>
-          <t>21,955,422</t>
+          <t>1,669,243</t>
         </is>
       </c>
       <c r="P28" s="5" t="n"/>
       <c r="Q28" s="28" t="inlineStr">
         <is>
-          <t>21,955,422</t>
+          <t>1,707,145</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>40,000</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>40,000</t>
         </is>
       </c>
     </row>
@@ -2132,9 +2285,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="M29" s="28" t="inlineStr">
-        <is>
-          <t>YES, outstanding: 1,451,424, limit: 1,500,000</t>
+      <c r="M29" s="133" t="inlineStr">
+        <is>
+          <t>NO, outstanding: 6,197,842, limit: 6,079,160</t>
         </is>
       </c>
       <c r="N29" s="5" t="n"/>
@@ -2145,6 +2298,16 @@
       </c>
       <c r="P29" s="5" t="n"/>
       <c r="Q29" s="24" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -2170,19 +2333,29 @@
       </c>
       <c r="M30" s="28" t="inlineStr">
         <is>
-          <t>16: YES, outstanding: 15,520,690, limit: 17,714,987</t>
+          <t>YES, outstanding: 30,667,835, limit: 34,070,376</t>
         </is>
       </c>
       <c r="N30" s="5" t="n"/>
       <c r="O30" s="24" t="inlineStr">
         <is>
-          <t>10: YES, outstanding: 1,753,657, limit: 2,146,309</t>
+          <t>YES, outstanding: 1,349,839, limit: 1,669,243</t>
         </is>
       </c>
       <c r="P30" s="5" t="n"/>
       <c r="Q30" s="24" t="inlineStr">
         <is>
-          <t>9: YES, outstanding: 1,723,015, limit: 2,094,126</t>
+          <t>YES, outstanding: 1,278,562, limit: 1,707,145</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>YES, outstanding: 17,053, limit: 40,000</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>YES, outstanding: 17,053, limit: 40,000</t>
         </is>
       </c>
     </row>
@@ -2204,21 +2377,31 @@
           <t>&gt; 2 times MIA2 for past 6 months and /or current 1 month &gt; 4 times MIA1</t>
         </is>
       </c>
-      <c r="M31" s="27" t="inlineStr">
-        <is>
-          <t>past 6 months MIA1: 1, MIA2: 0, MIA3: 0, MIA4+: 0 and /or current 1 month MIA1: 1, MIA2: 0, MIA3: 0, MIA4+: 0</t>
+      <c r="M31" s="131" t="inlineStr">
+        <is>
+          <t>past 6 months MIA1: 61, MIA2: 0, MIA3: 2, MIA4+: 0 and /or current 1 month MIA1: 34, MIA2: 0, MIA3: 1, MIA4+: 0</t>
         </is>
       </c>
       <c r="N31" s="5" t="n"/>
-      <c r="O31" s="131" t="inlineStr">
-        <is>
-          <t>past 6 months MIA1: 1, MIA2: 1, MIA3: 1, MIA4+: 2 and /or current 1 month MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 1</t>
+      <c r="O31" s="27" t="inlineStr">
+        <is>
+          <t>past 6 months MIA1: 10, MIA2: 1, MIA3: 0, MIA4+: 0 and /or current 1 month MIA1: 4, MIA2: 0, MIA3: 0, MIA4+: 0</t>
         </is>
       </c>
       <c r="P31" s="5" t="n"/>
-      <c r="Q31" s="131" t="inlineStr">
-        <is>
-          <t>past 6 months MIA1: 6, MIA2: 3, MIA3: 1, MIA4+: 0 and /or current 1 month MIA1: 0, MIA2: 1, MIA3: 0, MIA4+: 0</t>
+      <c r="Q31" s="27" t="inlineStr">
+        <is>
+          <t>past 6 months MIA1: 8, MIA2: 0, MIA3: 0, MIA4+: 0 and /or current 1 month MIA1: 1, MIA2: 0, MIA3: 0, MIA4+: 0</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>past 6 months MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 0 and /or current 1 month MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 0</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>past 6 months MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 0 and /or current 1 month MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 0</t>
         </is>
       </c>
     </row>
@@ -2257,6 +2440,16 @@
           <t>N/A</t>
         </is>
       </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="42" customFormat="1" customHeight="1" s="2">
       <c r="D33" s="115" t="inlineStr">
@@ -2276,19 +2469,29 @@
           <t>No</t>
         </is>
       </c>
-      <c r="M33" s="132" t="inlineStr">
+      <c r="M33" s="133" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
       <c r="N33" s="5" t="n"/>
-      <c r="O33" s="133" t="inlineStr">
+      <c r="O33" s="134" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
       <c r="P33" s="5" t="n"/>
-      <c r="Q33" s="133" t="inlineStr">
+      <c r="Q33" s="134" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="S33" s="132" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="U33" s="132" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -2312,21 +2515,31 @@
           <t>&gt; 2 times MIA2 for past 6 months and /or current 1 month &gt; 4 times MIA1</t>
         </is>
       </c>
-      <c r="M34" s="27" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="M34" s="131" t="inlineStr">
+        <is>
+          <t>past 6 months MIA1: 2, MIA2: 4, MIA3: 2, MIA4+: 4 and /or current 1 month MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 2</t>
         </is>
       </c>
       <c r="N34" s="5" t="n"/>
-      <c r="O34" s="27" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="O34" s="131" t="inlineStr">
+        <is>
+          <t>past 6 months MIA1: 2, MIA2: 4, MIA3: 2, MIA4+: 4 and /or current 1 month MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 2</t>
         </is>
       </c>
       <c r="P34" s="5" t="n"/>
-      <c r="Q34" s="27" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="Q34" s="131" t="inlineStr">
+        <is>
+          <t>past 6 months MIA1: 2, MIA2: 4, MIA3: 2, MIA4+: 4 and /or current 1 month MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 2</t>
+        </is>
+      </c>
+      <c r="S34" s="132" t="inlineStr">
+        <is>
+          <t>past 6 months MIA1: 2, MIA2: 4, MIA3: 2, MIA4+: 4 and /or current 1 month MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 2</t>
+        </is>
+      </c>
+      <c r="U34" s="132" t="inlineStr">
+        <is>
+          <t>past 6 months MIA1: 2, MIA2: 4, MIA3: 2, MIA4+: 4 and /or current 1 month MIA1: 0, MIA2: 0, MIA3: 0, MIA4+: 2</t>
         </is>
       </c>
     </row>
@@ -2350,19 +2563,29 @@
       </c>
       <c r="M35" s="129" t="inlineStr">
         <is>
-          <t>WITHDRAWN</t>
+          <t>LOD</t>
         </is>
       </c>
       <c r="N35" s="5" t="n"/>
       <c r="O35" s="131" t="inlineStr">
         <is>
-          <t>WITHDRAWN</t>
+          <t>LOD</t>
         </is>
       </c>
       <c r="P35" s="5" t="n"/>
       <c r="Q35" s="131" t="inlineStr">
         <is>
-          <t>WITHDRAWN</t>
+          <t>LOD</t>
+        </is>
+      </c>
+      <c r="S35" s="132" t="inlineStr">
+        <is>
+          <t>LOD</t>
+        </is>
+      </c>
+      <c r="U35" s="132" t="inlineStr">
+        <is>
+          <t>LOD</t>
         </is>
       </c>
     </row>
@@ -2577,7 +2800,7 @@
       <c r="L44" s="36" t="n"/>
     </row>
     <row r="45">
-      <c r="D45" s="134" t="n"/>
+      <c r="D45" s="135" t="n"/>
       <c r="H45" s="34" t="n"/>
       <c r="I45" s="35" t="n"/>
       <c r="J45" s="34" t="n"/>
@@ -2820,36 +3043,36 @@
     </row>
     <row r="58" ht="17.1" customFormat="1" customHeight="1" s="36">
       <c r="C58" s="58" t="n"/>
-      <c r="D58" s="135" t="inlineStr">
+      <c r="D58" s="136" t="inlineStr">
         <is>
           <t>By Credit Analyst</t>
         </is>
       </c>
-      <c r="E58" s="136" t="n"/>
-      <c r="F58" s="135" t="inlineStr">
+      <c r="E58" s="137" t="n"/>
+      <c r="F58" s="136" t="inlineStr">
         <is>
           <t>Justifications:</t>
         </is>
       </c>
-      <c r="G58" s="137" t="n"/>
-      <c r="H58" s="137" t="n"/>
-      <c r="I58" s="137" t="n"/>
-      <c r="J58" s="137" t="n"/>
-      <c r="K58" s="136" t="n"/>
+      <c r="G58" s="138" t="n"/>
+      <c r="H58" s="138" t="n"/>
+      <c r="I58" s="138" t="n"/>
+      <c r="J58" s="138" t="n"/>
+      <c r="K58" s="137" t="n"/>
       <c r="L58" s="63" t="inlineStr">
         <is>
           <t>By Chief Credit Officer</t>
         </is>
       </c>
-      <c r="M58" s="135" t="inlineStr">
+      <c r="M58" s="136" t="inlineStr">
         <is>
           <t>Justifications:</t>
         </is>
       </c>
-      <c r="N58" s="137" t="n"/>
-      <c r="O58" s="137" t="n"/>
-      <c r="P58" s="137" t="n"/>
-      <c r="Q58" s="136" t="n"/>
+      <c r="N58" s="138" t="n"/>
+      <c r="O58" s="138" t="n"/>
+      <c r="P58" s="138" t="n"/>
+      <c r="Q58" s="137" t="n"/>
       <c r="R58" s="57" t="n"/>
       <c r="S58" s="1" t="n"/>
     </row>
@@ -3005,36 +3228,36 @@
     </row>
     <row r="67" ht="14.25" customFormat="1" customHeight="1" s="36">
       <c r="C67" s="58" t="n"/>
-      <c r="D67" s="135" t="inlineStr">
+      <c r="D67" s="136" t="inlineStr">
         <is>
           <t>By Credit Committee 1</t>
         </is>
       </c>
-      <c r="E67" s="136" t="n"/>
-      <c r="F67" s="135" t="inlineStr">
+      <c r="E67" s="137" t="n"/>
+      <c r="F67" s="136" t="inlineStr">
         <is>
           <t>Justifications:</t>
         </is>
       </c>
-      <c r="G67" s="137" t="n"/>
-      <c r="H67" s="137" t="n"/>
-      <c r="I67" s="137" t="n"/>
-      <c r="J67" s="137" t="n"/>
-      <c r="K67" s="136" t="n"/>
+      <c r="G67" s="138" t="n"/>
+      <c r="H67" s="138" t="n"/>
+      <c r="I67" s="138" t="n"/>
+      <c r="J67" s="138" t="n"/>
+      <c r="K67" s="137" t="n"/>
       <c r="L67" s="78" t="inlineStr">
         <is>
           <t>By Credit Committee 2</t>
         </is>
       </c>
-      <c r="M67" s="135" t="inlineStr">
+      <c r="M67" s="136" t="inlineStr">
         <is>
           <t>Justifications:</t>
         </is>
       </c>
-      <c r="N67" s="137" t="n"/>
-      <c r="O67" s="137" t="n"/>
-      <c r="P67" s="137" t="n"/>
-      <c r="Q67" s="136" t="n"/>
+      <c r="N67" s="138" t="n"/>
+      <c r="O67" s="138" t="n"/>
+      <c r="P67" s="138" t="n"/>
+      <c r="Q67" s="137" t="n"/>
       <c r="R67" s="57" t="n"/>
       <c r="S67" s="1" t="n"/>
     </row>

</xml_diff>